<commit_message>
new liquid kristall design and kristall integration, including new scripts for UI checks and manual audits, as well as updates to existing files for improved functionality and user experience.
</commit_message>
<xml_diff>
--- a/Excel Template.xlsx
+++ b/Excel Template.xlsx
@@ -301,8 +301,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr defaultRowHeight="14.35" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" defaultColWidth="10.703125" customHeight="1"/>
+  <cols>
+    <col min="17" max="22" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -358,8 +361,35 @@
       <c r="P3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q3" s="1" t="s">
-        <v>11</v>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 1</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 2</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 3</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 4</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 5</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 6</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -380,6 +410,11 @@
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -400,6 +435,11 @@
       <c r="J6" s="1">
         <f t="shared" ref="J6:J30" si="1">IF(COUNT(B6:G6)=0,"",ROUND(I6,1))</f>
       </c>
+      <c r="R6"/>
+      <c r="S6"/>
+      <c r="T6"/>
+      <c r="U6"/>
+      <c r="V6"/>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -420,6 +460,11 @@
       <c r="J7" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R7"/>
+      <c r="S7"/>
+      <c r="T7"/>
+      <c r="U7"/>
+      <c r="V7"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -440,6 +485,11 @@
       <c r="J8" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -460,6 +510,11 @@
       <c r="J9" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R9"/>
+      <c r="S9"/>
+      <c r="T9"/>
+      <c r="U9"/>
+      <c r="V9"/>
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -480,6 +535,11 @@
       <c r="J10" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R10"/>
+      <c r="S10"/>
+      <c r="T10"/>
+      <c r="U10"/>
+      <c r="V10"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
@@ -493,6 +553,11 @@
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
+      <c r="R11"/>
+      <c r="S11"/>
+      <c r="T11"/>
+      <c r="U11"/>
+      <c r="V11"/>
     </row>
     <row r="12" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
@@ -506,6 +571,11 @@
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12"/>
+      <c r="U12"/>
+      <c r="V12"/>
     </row>
     <row r="13" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
@@ -519,6 +589,11 @@
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13"/>
+      <c r="U13"/>
+      <c r="V13"/>
     </row>
     <row r="14" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
@@ -532,6 +607,11 @@
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14"/>
+      <c r="U14"/>
+      <c r="V14"/>
     </row>
     <row r="15" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
@@ -545,6 +625,11 @@
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15"/>
+      <c r="V15"/>
     </row>
     <row r="16" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
@@ -558,6 +643,11 @@
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16"/>
+      <c r="V16"/>
     </row>
     <row r="17" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
@@ -571,6 +661,11 @@
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17"/>
+      <c r="V17"/>
     </row>
     <row r="18" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
@@ -584,6 +679,11 @@
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
     </row>
     <row r="19" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
@@ -597,6 +697,11 @@
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19"/>
+      <c r="V19"/>
     </row>
     <row r="20" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
@@ -610,6 +715,11 @@
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
     </row>
     <row r="21" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
@@ -623,6 +733,11 @@
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
     </row>
     <row r="22" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
@@ -636,6 +751,11 @@
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+      <c r="U22"/>
+      <c r="V22"/>
     </row>
     <row r="23" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
@@ -649,6 +769,11 @@
       </c>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
     </row>
     <row r="24" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
@@ -662,6 +787,11 @@
       </c>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+      <c r="U24"/>
+      <c r="V24"/>
     </row>
     <row r="25" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
@@ -675,6 +805,11 @@
       </c>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25"/>
+      <c r="U25"/>
+      <c r="V25"/>
     </row>
     <row r="26" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
@@ -688,6 +823,11 @@
       </c>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26"/>
+      <c r="V26"/>
     </row>
     <row r="27" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
@@ -701,6 +841,11 @@
       </c>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+      <c r="U27"/>
+      <c r="V27"/>
     </row>
     <row r="28" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
@@ -714,6 +859,11 @@
       </c>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
     </row>
     <row r="29" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
@@ -727,6 +877,11 @@
       </c>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
+      <c r="R29"/>
+      <c r="S29"/>
+      <c r="T29"/>
+      <c r="U29"/>
+      <c r="V29"/>
     </row>
     <row r="30" ht="15" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
@@ -740,9 +895,14 @@
       </c>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
+      <c r="R30"/>
+      <c r="S30"/>
+      <c r="T30"/>
+      <c r="U30"/>
+      <c r="V30"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="22">
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
@@ -760,6 +920,11 @@
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
     <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="V3:V4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -768,8 +933,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr defaultRowHeight="14.35" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" defaultColWidth="10.703125" customHeight="1"/>
+  <cols>
+    <col min="17" max="22" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -825,8 +993,35 @@
       <c r="P3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q3" s="1" t="s">
-        <v>11</v>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 1</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 2</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 3</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 4</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 5</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 6</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -847,6 +1042,11 @@
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -867,6 +1067,11 @@
       <c r="J6" s="1">
         <f t="shared" ref="J6:J30" si="1">IF(COUNT(B6:G6)=0,"",ROUND(I6,1))</f>
       </c>
+      <c r="R6"/>
+      <c r="S6"/>
+      <c r="T6"/>
+      <c r="U6"/>
+      <c r="V6"/>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -887,6 +1092,11 @@
       <c r="J7" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R7"/>
+      <c r="S7"/>
+      <c r="T7"/>
+      <c r="U7"/>
+      <c r="V7"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -907,6 +1117,11 @@
       <c r="J8" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -927,6 +1142,11 @@
       <c r="J9" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R9"/>
+      <c r="S9"/>
+      <c r="T9"/>
+      <c r="U9"/>
+      <c r="V9"/>
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -947,6 +1167,11 @@
       <c r="J10" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R10"/>
+      <c r="S10"/>
+      <c r="T10"/>
+      <c r="U10"/>
+      <c r="V10"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -967,6 +1192,11 @@
       <c r="J11" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R11"/>
+      <c r="S11"/>
+      <c r="T11"/>
+      <c r="U11"/>
+      <c r="V11"/>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -987,6 +1217,11 @@
       <c r="J12" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12"/>
+      <c r="U12"/>
+      <c r="V12"/>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1007,6 +1242,11 @@
       <c r="J13" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13"/>
+      <c r="U13"/>
+      <c r="V13"/>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1027,6 +1267,11 @@
       <c r="J14" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14"/>
+      <c r="U14"/>
+      <c r="V14"/>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1047,6 +1292,11 @@
       <c r="J15" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15"/>
+      <c r="V15"/>
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1067,6 +1317,11 @@
       <c r="J16" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16"/>
+      <c r="V16"/>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1087,6 +1342,11 @@
       <c r="J17" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17"/>
+      <c r="V17"/>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1107,6 +1367,11 @@
       <c r="J18" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1127,6 +1392,11 @@
       <c r="J19" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19"/>
+      <c r="V19"/>
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1147,6 +1417,11 @@
       <c r="J20" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1167,6 +1442,11 @@
       <c r="J21" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1187,6 +1467,11 @@
       <c r="J22" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+      <c r="U22"/>
+      <c r="V22"/>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -1207,6 +1492,11 @@
       <c r="J23" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -1227,6 +1517,11 @@
       <c r="J24" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+      <c r="U24"/>
+      <c r="V24"/>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1247,6 +1542,11 @@
       <c r="J25" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25"/>
+      <c r="U25"/>
+      <c r="V25"/>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1267,6 +1567,11 @@
       <c r="J26" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26"/>
+      <c r="V26"/>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1287,6 +1592,11 @@
       <c r="J27" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+      <c r="U27"/>
+      <c r="V27"/>
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -1307,6 +1617,11 @@
       <c r="J28" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1327,6 +1642,11 @@
       <c r="J29" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R29"/>
+      <c r="S29"/>
+      <c r="T29"/>
+      <c r="U29"/>
+      <c r="V29"/>
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -1347,9 +1667,14 @@
       <c r="J30" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R30"/>
+      <c r="S30"/>
+      <c r="T30"/>
+      <c r="U30"/>
+      <c r="V30"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="22">
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
@@ -1367,6 +1692,11 @@
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
     <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="V3:V4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -1375,8 +1705,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr defaultRowHeight="14.35" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.5" defaultColWidth="10.703125" customHeight="1"/>
+  <cols>
+    <col min="17" max="22" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1432,8 +1765,35 @@
       <c r="P3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q3" s="1" t="s">
-        <v>11</v>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 1</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 2</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 3</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 4</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 5</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>Joker Datum 6</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -1454,6 +1814,11 @@
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -1474,6 +1839,11 @@
       <c r="J6" s="1">
         <f t="shared" ref="J6:J30" si="1">IF(COUNT(B6:G6)=0,"",ROUND(I6,1))</f>
       </c>
+      <c r="R6"/>
+      <c r="S6"/>
+      <c r="T6"/>
+      <c r="U6"/>
+      <c r="V6"/>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1494,6 +1864,11 @@
       <c r="J7" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R7"/>
+      <c r="S7"/>
+      <c r="T7"/>
+      <c r="U7"/>
+      <c r="V7"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1514,6 +1889,11 @@
       <c r="J8" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1534,6 +1914,11 @@
       <c r="J9" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R9"/>
+      <c r="S9"/>
+      <c r="T9"/>
+      <c r="U9"/>
+      <c r="V9"/>
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1554,6 +1939,11 @@
       <c r="J10" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R10"/>
+      <c r="S10"/>
+      <c r="T10"/>
+      <c r="U10"/>
+      <c r="V10"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1574,6 +1964,11 @@
       <c r="J11" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R11"/>
+      <c r="S11"/>
+      <c r="T11"/>
+      <c r="U11"/>
+      <c r="V11"/>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1594,6 +1989,11 @@
       <c r="J12" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12"/>
+      <c r="U12"/>
+      <c r="V12"/>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1614,6 +2014,11 @@
       <c r="J13" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13"/>
+      <c r="U13"/>
+      <c r="V13"/>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1634,6 +2039,11 @@
       <c r="J14" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14"/>
+      <c r="U14"/>
+      <c r="V14"/>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1654,6 +2064,11 @@
       <c r="J15" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15"/>
+      <c r="V15"/>
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1674,6 +2089,11 @@
       <c r="J16" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16"/>
+      <c r="V16"/>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1694,6 +2114,11 @@
       <c r="J17" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17"/>
+      <c r="V17"/>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1714,6 +2139,11 @@
       <c r="J18" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1734,6 +2164,11 @@
       <c r="J19" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19"/>
+      <c r="V19"/>
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1754,6 +2189,11 @@
       <c r="J20" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1774,6 +2214,11 @@
       <c r="J21" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1794,6 +2239,11 @@
       <c r="J22" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+      <c r="U22"/>
+      <c r="V22"/>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -1814,6 +2264,11 @@
       <c r="J23" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -1834,6 +2289,11 @@
       <c r="J24" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+      <c r="U24"/>
+      <c r="V24"/>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1854,6 +2314,11 @@
       <c r="J25" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25"/>
+      <c r="U25"/>
+      <c r="V25"/>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1874,6 +2339,11 @@
       <c r="J26" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26"/>
+      <c r="V26"/>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1894,6 +2364,11 @@
       <c r="J27" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+      <c r="U27"/>
+      <c r="V27"/>
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -1914,6 +2389,11 @@
       <c r="J28" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1934,6 +2414,11 @@
       <c r="J29" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R29"/>
+      <c r="S29"/>
+      <c r="T29"/>
+      <c r="U29"/>
+      <c r="V29"/>
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -1954,9 +2439,14 @@
       <c r="J30" s="1">
         <f t="shared" si="1"/>
       </c>
+      <c r="R30"/>
+      <c r="S30"/>
+      <c r="T30"/>
+      <c r="U30"/>
+      <c r="V30"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="22">
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
@@ -1974,6 +2464,11 @@
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
     <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="V3:V4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>